<commit_message>
Honoraria: 5% per debater from Y2 onwards
Y1 unchanged (flat \$10K per bout). Y2 and Y3 honorarium pool rises
from a combined 5% / 3% of bout purse to 10% per bout (5% per each
of the two debaters). Aligns debater incentives with audience scale
and matches the "league pays its talent" narrative — the bigger the
purse, the bigger the take.

Annual honoraria spend (aggressive case):
  Y1   24 × \$10,000     = \$240K  (unchanged)
  Y2   48 × \$5,000      = \$240K  (was \$120K · +\$120K)
  Y3   48 × \$7,500      = \$360K  (was \$108K · +\$252K)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Argumental/argumental-app/public/argumental-financial-model.xlsx
+++ b/Argumental/argumental-app/public/argumental-financial-model.xlsx
@@ -1215,16 +1215,16 @@
         <v>10000</v>
       </c>
       <c r="C22" s="16">
-        <f>C8*C9*C10*0.05</f>
+        <f>C8*C9*C10*0.1</f>
         <v/>
       </c>
       <c r="D22" s="16">
-        <f>D8*D9*D10*0.03</f>
+        <f>D8*D9*D10*0.1</f>
         <v/>
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>Y1 flat $10,000 · Y2 5% · Y3 3% of purse</t>
+          <t>Y1 flat $10,000 · Y2 10% · Y3 10% of purse</t>
         </is>
       </c>
     </row>

</xml_diff>